<commit_message>
Feature: Transition to Hybrid Architecture with static templates and modular AI comments
</commit_message>
<xml_diff>
--- a/Bao cao/GMD/GMD_Model_2026-06.xlsx
+++ b/Bao cao/GMD/GMD_Model_2026-06.xlsx
@@ -7,8 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="P&amp;L" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="01_Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="02_Assumptions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="03_PnL" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="04_Ratios" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="#,##0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -27,14 +32,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
-      <sz val="18"/>
+      <color rgb="001A365D"/>
+      <sz val="16"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <i val="1"/>
-      <sz val="12"/>
+      <color rgb="004A5568"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -57,11 +64,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,41 +437,52 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:B6"/>
+  <dimension ref="B2:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>BÁO CÁO PHÂN TÍCH CỔ PHIẾU GMD</t>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>MÔ HÌNH PHÂN TÍCH TÀI CHÍNH &amp; ĐỊNH GIÁ GMD</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Công ty Cổ phần GMD</t>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Công ty Cổ phần Tập đoàn Gemadept</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Giá hiện tại:</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="C5" s="3" t="n">
         <v>10000</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Vốn hóa (tỷ):</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>10</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Số lượng CP lưu hành:</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>10000000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Vốn hóa thị trường (tỷ):</t>
+        </is>
+      </c>
+      <c r="C7" s="4">
+        <f>C5*C6/1000000000</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -475,178 +496,466 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Chỉ tiêu</t>
+          <t>Tham số giả định</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2021A</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>2022A</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>2023A</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>2024A</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>2025A</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>2026E</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>2027E</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>2028E</t>
+          <t>Giá trị</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Doanh thu thuần (tỷ)</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>3206.290165333</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>3898.24360857</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>3845.826296568</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>4832.024798961</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>5956.025297015</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <v>6849.42909156725</v>
-      </c>
-      <c r="H2" s="3" t="n">
-        <v>7876.843455302337</v>
-      </c>
-      <c r="I2" s="3" t="n">
-        <v>9058.369973597686</v>
+          <t>Tốc độ tăng trưởng DT dài hạn (g)</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>0.1728532740831309</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lợi nhuận gộp (tỷ)</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>1141.800934694</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>1718.060577087</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>1778.015187303</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>2135.48039702</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>2739.47253893</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>2960.399842290913</v>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>3404.459818634549</v>
-      </c>
-      <c r="I3" s="3" t="n">
-        <v>3915.128791429731</v>
+          <t>Biên lợi nhuận ròng dự báo</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lợi nhuận sau thuế (tỷ)</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>612.182073397</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>993.915564733</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>2250.57733992</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>1455.479595602</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>1755.629825296</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>2228.909847731341</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>2563.246324891042</v>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>2947.733273624698</v>
+          <t>P/E Mục tiêu</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>P/B Mục tiêu</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Số lượng cổ phiếu</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>10000000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Chỉ tiêu P&amp;L (tỷ VND)</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2021A</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>2022A</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>2023A</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>2024A</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>2025A</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>2027E</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Doanh thu thuần</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>3206.290165333</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>3898.24360857</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>3845.826296568</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>4832.024798961</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>5956.025297015</v>
+      </c>
+      <c r="G2" s="4">
+        <f>F2*(1+'02_Assumptions'!$B$2)</f>
+        <v/>
+      </c>
+      <c r="H2" s="4">
+        <f>G2*(1+'02_Assumptions'!$B$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Giá vốn hàng bán</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>2064.489230639</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>2180.183031483</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>2067.811109265</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>2696.544401941</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>3216.552758085</v>
+      </c>
+      <c r="G3" s="4">
+        <f>G2*0.75</f>
+        <v/>
+      </c>
+      <c r="H3" s="4">
+        <f>H2*0.75</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lợi nhuận gộp</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>1141.800934694</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>1718.060577087</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>1778.015187303</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>2135.48039702</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>2739.472538930001</v>
+      </c>
+      <c r="G4" s="4">
+        <f>G2-G3</f>
+        <v/>
+      </c>
+      <c r="H4" s="4">
+        <f>H2-H3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Lợi nhuận sau thuế (LNST)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>612.182073397</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>993.915564733</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>2250.57733992</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>1455.479595602</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>1755.629825296</v>
+      </c>
+      <c r="G5" s="4">
+        <f>G2*'02_Assumptions'!$B$3</f>
+        <v/>
+      </c>
+      <c r="H5" s="4">
+        <f>H2*'02_Assumptions'!$B$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>EPS (VND)</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B6" s="3" t="n">
         <v>1869</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C6" s="3" t="n">
         <v>3034</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D6" s="3" t="n">
         <v>7207</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E6" s="3" t="n">
         <v>4276</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F6" s="3" t="n">
         <v>3839</v>
       </c>
-      <c r="G5" s="3" t="n">
-        <v>2228909.847731341</v>
-      </c>
-      <c r="H5" s="3" t="n">
-        <v>2563246.324891041</v>
-      </c>
-      <c r="I5" s="3" t="n">
-        <v>2947733.273624698</v>
+      <c r="G6" s="3">
+        <f>G5*1000000000/'02_Assumptions'!$B$6</f>
+        <v/>
+      </c>
+      <c r="H6" s="3">
+        <f>H5*1000000000/'02_Assumptions'!$B$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Vốn chủ sở hữu (VCSH)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4">
+        <f>F7+G5*0.7</f>
+        <v/>
+      </c>
+      <c r="H7" s="4">
+        <f>G7+H5*0.7</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Chỉ số tài chính</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2021A</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>2022A</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>2023A</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>2024A</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>2025A</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>2027E</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Biên lợi nhuận gộp (%)</t>
+        </is>
+      </c>
+      <c r="B2" s="5">
+        <f>'03_PnL'!B4/'03_PnL'!B2</f>
+        <v/>
+      </c>
+      <c r="C2" s="5">
+        <f>'03_PnL'!C4/'03_PnL'!C2</f>
+        <v/>
+      </c>
+      <c r="D2" s="5">
+        <f>'03_PnL'!D4/'03_PnL'!D2</f>
+        <v/>
+      </c>
+      <c r="E2" s="5">
+        <f>'03_PnL'!E4/'03_PnL'!E2</f>
+        <v/>
+      </c>
+      <c r="F2" s="5">
+        <f>'03_PnL'!F4/'03_PnL'!F2</f>
+        <v/>
+      </c>
+      <c r="G2" s="5">
+        <f>'03_PnL'!G4/'03_PnL'!G2</f>
+        <v/>
+      </c>
+      <c r="H2" s="5">
+        <f>'03_PnL'!H4/'03_PnL'!H2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Biên lợi nhuận ròng (%)</t>
+        </is>
+      </c>
+      <c r="B3" s="5">
+        <f>'03_PnL'!B5/'03_PnL'!B2</f>
+        <v/>
+      </c>
+      <c r="C3" s="5">
+        <f>'03_PnL'!C5/'03_PnL'!C2</f>
+        <v/>
+      </c>
+      <c r="D3" s="5">
+        <f>'03_PnL'!D5/'03_PnL'!D2</f>
+        <v/>
+      </c>
+      <c r="E3" s="5">
+        <f>'03_PnL'!E5/'03_PnL'!E2</f>
+        <v/>
+      </c>
+      <c r="F3" s="5">
+        <f>'03_PnL'!F5/'03_PnL'!F2</f>
+        <v/>
+      </c>
+      <c r="G3" s="5">
+        <f>'03_PnL'!G5/'03_PnL'!G2</f>
+        <v/>
+      </c>
+      <c r="H3" s="5">
+        <f>'03_PnL'!H5/'03_PnL'!H2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Hiệu suất sử dụng vốn (ROE)</t>
+        </is>
+      </c>
+      <c r="B4" s="5">
+        <f>'03_PnL'!B5/'03_PnL'!B7</f>
+        <v/>
+      </c>
+      <c r="C4" s="5">
+        <f>'03_PnL'!C5/'03_PnL'!C7</f>
+        <v/>
+      </c>
+      <c r="D4" s="5">
+        <f>'03_PnL'!D5/'03_PnL'!D7</f>
+        <v/>
+      </c>
+      <c r="E4" s="5">
+        <f>'03_PnL'!E5/'03_PnL'!E7</f>
+        <v/>
+      </c>
+      <c r="F4" s="5">
+        <f>'03_PnL'!F5/'03_PnL'!F7</f>
+        <v/>
+      </c>
+      <c r="G4" s="5">
+        <f>'03_PnL'!G5/'03_PnL'!G7</f>
+        <v/>
+      </c>
+      <c r="H4" s="5">
+        <f>'03_PnL'!H5/'03_PnL'!H7</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>